<commit_message>
Selenium pytest third day commit
</commit_message>
<xml_diff>
--- a/SeleniumPytest/IxigoTripPlanner/testdata/testdata.xlsx
+++ b/SeleniumPytest/IxigoTripPlanner/testdata/testdata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WiproCapstone\SeleniumPytest\IxigoTripPlanner\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{808D0C45-3EB1-4812-B226-6BE86FD6375C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D617F37-F482-479E-B2F2-9F481C1DD45F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1404" yWindow="672" windowWidth="15336" windowHeight="11688" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1404" yWindow="672" windowWidth="15336" windowHeight="11688" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PlannerData" sheetId="1" r:id="rId1"/>
@@ -132,9 +132,6 @@
     <t>Denpasar</t>
   </si>
   <si>
-    <t>Kuala Lumpur</t>
-  </si>
-  <si>
     <t>Sumatra</t>
   </si>
   <si>
@@ -679,6 +676,9 @@
   </si>
   <si>
     <t>islands</t>
+  </si>
+  <si>
+    <t>Hikone</t>
   </si>
 </sst>
 </file>
@@ -1175,7 +1175,7 @@
         <v>28</v>
       </c>
       <c r="C2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -1186,7 +1186,7 @@
         <v>29</v>
       </c>
       <c r="C3" t="s">
-        <v>34</v>
+        <v>216</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -1197,15 +1197,15 @@
         <v>30</v>
       </c>
       <c r="C4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -1213,7 +1213,7 @@
         <v>31</v>
       </c>
       <c r="C6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -1226,102 +1226,102 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C10" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C12" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C13" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C14" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C16" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="17" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C17" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="18" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C18" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="19" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C19" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="20" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C20" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="21" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C21" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="22" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C22" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="23" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C23" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="24" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C24" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="25" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="26" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C26" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="27" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C27" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="28" spans="3:3" x14ac:dyDescent="0.3">
@@ -1331,772 +1331,772 @@
     </row>
     <row r="29" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C29" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="30" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C30" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="31" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C31" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="32" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C32" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="33" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C33" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="34" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C34" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="35" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C35" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="36" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C36" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="37" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C37" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="38" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C38" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="39" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C39" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="40" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C40" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="41" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C41" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="42" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C42" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="43" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C43" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="44" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C44" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="45" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C45" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="46" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C46" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="47" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C47" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="48" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C48" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="49" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C49" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="50" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C50" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="51" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C51" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="52" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C52" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="53" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C53" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="54" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C54" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="55" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C55" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="56" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C56" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="57" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C57" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="58" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C58" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="59" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C59" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="60" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C60" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="61" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C61" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="62" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C62" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="63" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C63" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="64" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C64" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="65" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C65" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="66" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C66" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="67" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C67" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="68" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C68" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="69" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C69" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="70" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C70" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="71" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C71" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="72" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C72" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="73" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C73" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="74" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C74" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="75" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C75" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="76" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C76" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="77" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C77" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="78" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C78" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="79" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C79" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="80" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C80" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="81" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C81" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="82" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C82" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="83" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C83" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="84" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C84" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="85" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C85" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="86" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C86" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="87" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C87" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="88" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C88" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="89" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C89" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="90" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C90" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="91" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C91" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="92" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C92" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="93" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C93" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="94" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C94" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="95" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C95" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="96" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C96" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="97" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C97" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="98" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C98" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="99" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C99" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="100" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C100" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="101" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C101" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="102" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C102" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="103" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C103" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="104" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C104" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="105" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C105" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="106" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C106" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="107" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C107" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="108" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C108" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="109" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C109" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="110" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C110" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="111" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C111" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="112" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C112" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="113" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C113" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="114" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C114" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="115" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C115" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="116" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C116" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="117" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C117" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="118" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C118" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="119" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C119" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="120" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C120" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="121" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C121" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="122" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C122" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="123" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C123" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="124" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C124" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="125" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C125" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="126" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C126" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="127" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C127" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="128" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C128" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="129" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C129" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="130" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C130" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="131" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C131" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="132" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C132" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="133" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C133" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="134" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C134" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="135" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C135" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="136" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C136" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="137" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C137" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="138" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C138" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="139" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C139" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="140" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C140" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="141" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C141" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="142" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C142" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="143" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C143" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="144" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C144" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="145" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C145" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="146" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C146" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="147" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C147" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="148" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C148" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="149" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C149" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="150" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C150" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="151" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C151" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="152" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C152" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="153" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C153" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="154" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C154" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="155" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C155" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="156" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C156" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="157" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C157" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="158" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C158" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="159" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C159" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="160" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C160" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="161" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C161" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="162" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C162" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="163" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C163" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="164" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C164" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="165" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C165" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="166" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C166" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="167" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C167" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="168" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C168" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="169" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C169" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="170" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C170" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="171" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C171" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="172" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C172" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="173" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C173" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="174" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C174" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="175" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C175" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="176" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C176" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="177" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C177" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="178" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C178" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="179" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C179" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="180" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C180" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="181" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C181" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="182" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C182" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
   </sheetData>
@@ -2118,40 +2118,40 @@
         <v>24</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Selenium pytest Final day commit
</commit_message>
<xml_diff>
--- a/SeleniumPytest/IxigoTripPlanner/testdata/testdata.xlsx
+++ b/SeleniumPytest/IxigoTripPlanner/testdata/testdata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WiproCapstone\SeleniumPytest\IxigoTripPlanner\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D617F37-F482-479E-B2F2-9F481C1DD45F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3967EAE1-6241-455F-87D4-362B1BEA2ECB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1404" yWindow="672" windowWidth="15336" windowHeight="11688" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-48" yWindow="-48" windowWidth="23136" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PlannerData" sheetId="1" r:id="rId1"/>

</xml_diff>